<commit_message>
added NSs mutant pMDS numbers to the metadata file
</commit_message>
<xml_diff>
--- a/2025_01_14_MG_LACV_50N_1/2025_01_17_LACV_50N_exp1_tidy.xlsx
+++ b/2025_01_14_MG_LACV_50N_1/2025_01_17_LACV_50N_exp1_tidy.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charligeer/Documents/Lab_Projects/MG_Assays/2025.01.14_MG_LACV_50N_1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charligeer/Documents/Lab_Projects/Repos/Bunya-50-N-experiments/2025_01_14_MG_LACV_50N_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C38E941-D710-1140-B3B4-7818DFEEC011}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABC39E51-C3BE-0743-9CB4-60576340FE1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="42020" yWindow="2420" windowWidth="24600" windowHeight="22700" xr2:uid="{CD6AA7B1-C22D-8C4D-94EB-7BEC7C6477A9}"/>
   </bookViews>
@@ -59,9 +59,6 @@
     <t>replicate</t>
   </si>
   <si>
-    <t>Experimen t</t>
-  </si>
-  <si>
     <t>none</t>
   </si>
   <si>
@@ -225,6 +222,9 @@
   </si>
   <si>
     <t>Wyeomyia virus</t>
+  </si>
+  <si>
+    <t>Experiment</t>
   </si>
 </sst>
 </file>
@@ -800,7 +800,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>62</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -832,10 +832,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
         <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
       </c>
       <c r="E2">
         <v>169</v>
@@ -858,10 +858,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
         <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
       </c>
       <c r="E3">
         <v>169</v>
@@ -884,10 +884,10 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E4">
         <v>169</v>
@@ -910,10 +910,10 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E5">
         <v>59</v>
@@ -936,10 +936,10 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E6">
         <v>60</v>
@@ -962,10 +962,10 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E7">
         <v>61</v>
@@ -988,10 +988,10 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E8">
         <v>62</v>
@@ -1014,10 +1014,10 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E9">
         <v>63</v>
@@ -1040,10 +1040,10 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E10">
         <v>64</v>
@@ -1066,10 +1066,10 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E11">
         <v>65</v>
@@ -1092,10 +1092,10 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E12">
         <v>66</v>
@@ -1118,10 +1118,10 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E13">
         <v>67</v>
@@ -1144,10 +1144,10 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E14">
         <v>68</v>
@@ -1170,10 +1170,10 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E15">
         <v>69</v>
@@ -1196,10 +1196,10 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E16">
         <v>127</v>
@@ -1222,10 +1222,10 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E17">
         <v>163</v>
@@ -1248,10 +1248,10 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E18">
         <v>164</v>
@@ -1274,10 +1274,10 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E19">
         <v>165</v>
@@ -1300,10 +1300,10 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E20">
         <v>166</v>
@@ -1326,10 +1326,10 @@
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E21">
         <v>167</v>
@@ -1352,10 +1352,10 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E22">
         <v>170</v>
@@ -1378,10 +1378,10 @@
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E23">
         <v>219</v>
@@ -1404,10 +1404,10 @@
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E24">
         <v>221</v>
@@ -1430,10 +1430,10 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E25">
         <v>222</v>
@@ -1456,10 +1456,10 @@
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E26">
         <v>223</v>
@@ -1482,10 +1482,10 @@
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D27" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E27">
         <v>224</v>
@@ -1508,10 +1508,10 @@
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D28" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E28">
         <v>225</v>
@@ -1534,10 +1534,10 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D29" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E29">
         <v>226</v>
@@ -1560,10 +1560,10 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D30" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E30">
         <v>227</v>
@@ -1586,10 +1586,10 @@
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D31" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E31">
         <v>228</v>
@@ -1612,10 +1612,10 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E32">
         <v>229</v>
@@ -1638,10 +1638,10 @@
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D33" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E33">
         <v>230</v>
@@ -1664,10 +1664,10 @@
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D34" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E34">
         <v>231</v>
@@ -1690,10 +1690,10 @@
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D35" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E35">
         <v>232</v>
@@ -1716,10 +1716,10 @@
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E36">
         <v>233</v>
@@ -1742,10 +1742,10 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E37">
         <v>234</v>
@@ -1768,10 +1768,10 @@
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D38" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E38">
         <v>235</v>
@@ -1794,10 +1794,10 @@
         <v>1</v>
       </c>
       <c r="C39" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D39" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E39">
         <v>236</v>
@@ -1820,10 +1820,10 @@
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D40" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E40">
         <v>237</v>
@@ -1846,10 +1846,10 @@
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D41" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E41">
         <v>238</v>
@@ -1872,10 +1872,10 @@
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D42" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E42">
         <v>239</v>
@@ -1898,10 +1898,10 @@
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D43" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E43">
         <v>240</v>
@@ -1924,10 +1924,10 @@
         <v>1</v>
       </c>
       <c r="C44" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D44" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E44">
         <v>241</v>
@@ -1950,10 +1950,10 @@
         <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D45" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E45">
         <v>242</v>
@@ -1976,10 +1976,10 @@
         <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D46" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E46">
         <v>243</v>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D47" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E47">
         <v>244</v>
@@ -2028,10 +2028,10 @@
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D48" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E48">
         <v>245</v>
@@ -2054,10 +2054,10 @@
         <v>1</v>
       </c>
       <c r="C49" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E49">
         <v>246</v>
@@ -2080,10 +2080,10 @@
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D50" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E50">
         <v>247</v>
@@ -2106,10 +2106,10 @@
         <v>1</v>
       </c>
       <c r="C51" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D51" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E51">
         <v>248</v>
@@ -2132,10 +2132,10 @@
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D52" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E52">
         <v>249</v>
@@ -2158,10 +2158,10 @@
         <v>1</v>
       </c>
       <c r="C53" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D53" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E53">
         <v>250</v>
@@ -2184,10 +2184,10 @@
         <v>1</v>
       </c>
       <c r="C54" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D54" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E54">
         <v>251</v>
@@ -2210,10 +2210,10 @@
         <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D55" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E55">
         <v>169</v>
@@ -2236,10 +2236,10 @@
         <v>2</v>
       </c>
       <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56" t="s">
         <v>8</v>
-      </c>
-      <c r="D56" t="s">
-        <v>9</v>
       </c>
       <c r="E56">
         <v>169</v>
@@ -2262,10 +2262,10 @@
         <v>2</v>
       </c>
       <c r="C57" t="s">
+        <v>9</v>
+      </c>
+      <c r="D57" t="s">
         <v>10</v>
-      </c>
-      <c r="D57" t="s">
-        <v>11</v>
       </c>
       <c r="E57">
         <v>169</v>
@@ -2288,10 +2288,10 @@
         <v>2</v>
       </c>
       <c r="C58" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D58" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E58">
         <v>169</v>
@@ -2314,10 +2314,10 @@
         <v>2</v>
       </c>
       <c r="C59" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D59" s="23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E59">
         <v>59</v>
@@ -2340,10 +2340,10 @@
         <v>2</v>
       </c>
       <c r="C60" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D60" s="23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E60">
         <v>60</v>
@@ -2366,10 +2366,10 @@
         <v>2</v>
       </c>
       <c r="C61" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D61" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E61">
         <v>61</v>
@@ -2392,10 +2392,10 @@
         <v>2</v>
       </c>
       <c r="C62" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D62" s="23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E62">
         <v>62</v>
@@ -2418,10 +2418,10 @@
         <v>2</v>
       </c>
       <c r="C63" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D63" s="23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E63">
         <v>63</v>
@@ -2444,10 +2444,10 @@
         <v>2</v>
       </c>
       <c r="C64" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D64" s="23" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E64">
         <v>64</v>
@@ -2470,10 +2470,10 @@
         <v>2</v>
       </c>
       <c r="C65" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D65" s="23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E65">
         <v>65</v>
@@ -2496,10 +2496,10 @@
         <v>2</v>
       </c>
       <c r="C66" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D66" s="23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E66">
         <v>66</v>
@@ -2522,10 +2522,10 @@
         <v>2</v>
       </c>
       <c r="C67" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D67" s="23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E67">
         <v>67</v>
@@ -2548,10 +2548,10 @@
         <v>2</v>
       </c>
       <c r="C68" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D68" s="23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E68">
         <v>68</v>
@@ -2574,10 +2574,10 @@
         <v>2</v>
       </c>
       <c r="C69" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D69" s="23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E69">
         <v>69</v>
@@ -2600,10 +2600,10 @@
         <v>2</v>
       </c>
       <c r="C70" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D70" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E70">
         <v>127</v>
@@ -2626,10 +2626,10 @@
         <v>2</v>
       </c>
       <c r="C71" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D71" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E71">
         <v>163</v>
@@ -2652,10 +2652,10 @@
         <v>2</v>
       </c>
       <c r="C72" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D72" s="23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E72">
         <v>164</v>
@@ -2678,10 +2678,10 @@
         <v>2</v>
       </c>
       <c r="C73" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D73" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E73">
         <v>165</v>
@@ -2704,10 +2704,10 @@
         <v>2</v>
       </c>
       <c r="C74" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D74" s="23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E74">
         <v>166</v>
@@ -2730,10 +2730,10 @@
         <v>2</v>
       </c>
       <c r="C75" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E75">
         <v>167</v>
@@ -2756,10 +2756,10 @@
         <v>2</v>
       </c>
       <c r="C76" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E76">
         <v>170</v>
@@ -2782,10 +2782,10 @@
         <v>2</v>
       </c>
       <c r="C77" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E77">
         <v>219</v>
@@ -2808,10 +2808,10 @@
         <v>2</v>
       </c>
       <c r="C78" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D78" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E78">
         <v>221</v>
@@ -2834,10 +2834,10 @@
         <v>2</v>
       </c>
       <c r="C79" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D79" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E79">
         <v>222</v>
@@ -2860,10 +2860,10 @@
         <v>2</v>
       </c>
       <c r="C80" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D80" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E80">
         <v>223</v>
@@ -2886,10 +2886,10 @@
         <v>2</v>
       </c>
       <c r="C81" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D81" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E81">
         <v>224</v>
@@ -2912,10 +2912,10 @@
         <v>2</v>
       </c>
       <c r="C82" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D82" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E82">
         <v>225</v>
@@ -2938,10 +2938,10 @@
         <v>2</v>
       </c>
       <c r="C83" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D83" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E83">
         <v>226</v>
@@ -2964,10 +2964,10 @@
         <v>2</v>
       </c>
       <c r="C84" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D84" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E84">
         <v>227</v>
@@ -2990,10 +2990,10 @@
         <v>2</v>
       </c>
       <c r="C85" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D85" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E85">
         <v>228</v>
@@ -3016,10 +3016,10 @@
         <v>2</v>
       </c>
       <c r="C86" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D86" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E86">
         <v>229</v>
@@ -3042,10 +3042,10 @@
         <v>2</v>
       </c>
       <c r="C87" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D87" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E87">
         <v>230</v>
@@ -3068,10 +3068,10 @@
         <v>2</v>
       </c>
       <c r="C88" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D88" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E88">
         <v>231</v>
@@ -3094,10 +3094,10 @@
         <v>2</v>
       </c>
       <c r="C89" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D89" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E89">
         <v>232</v>
@@ -3120,10 +3120,10 @@
         <v>2</v>
       </c>
       <c r="C90" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D90" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E90">
         <v>233</v>
@@ -3146,10 +3146,10 @@
         <v>2</v>
       </c>
       <c r="C91" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D91" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E91">
         <v>234</v>
@@ -3172,10 +3172,10 @@
         <v>2</v>
       </c>
       <c r="C92" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D92" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E92">
         <v>235</v>
@@ -3198,10 +3198,10 @@
         <v>2</v>
       </c>
       <c r="C93" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D93" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E93">
         <v>236</v>
@@ -3224,10 +3224,10 @@
         <v>2</v>
       </c>
       <c r="C94" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D94" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E94">
         <v>237</v>
@@ -3250,10 +3250,10 @@
         <v>2</v>
       </c>
       <c r="C95" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D95" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E95">
         <v>238</v>
@@ -3276,10 +3276,10 @@
         <v>2</v>
       </c>
       <c r="C96" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D96" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E96">
         <v>239</v>
@@ -3302,10 +3302,10 @@
         <v>2</v>
       </c>
       <c r="C97" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D97" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E97">
         <v>240</v>
@@ -3328,10 +3328,10 @@
         <v>2</v>
       </c>
       <c r="C98" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D98" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E98">
         <v>241</v>
@@ -3354,10 +3354,10 @@
         <v>2</v>
       </c>
       <c r="C99" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D99" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E99">
         <v>242</v>
@@ -3380,10 +3380,10 @@
         <v>2</v>
       </c>
       <c r="C100" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D100" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E100">
         <v>243</v>
@@ -3406,10 +3406,10 @@
         <v>2</v>
       </c>
       <c r="C101" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D101" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E101">
         <v>244</v>
@@ -3432,10 +3432,10 @@
         <v>2</v>
       </c>
       <c r="C102" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D102" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E102">
         <v>245</v>
@@ -3458,10 +3458,10 @@
         <v>2</v>
       </c>
       <c r="C103" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D103" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E103">
         <v>246</v>
@@ -3484,10 +3484,10 @@
         <v>2</v>
       </c>
       <c r="C104" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D104" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E104">
         <v>247</v>
@@ -3510,10 +3510,10 @@
         <v>2</v>
       </c>
       <c r="C105" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D105" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E105">
         <v>248</v>
@@ -3536,10 +3536,10 @@
         <v>2</v>
       </c>
       <c r="C106" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D106" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E106">
         <v>249</v>
@@ -3562,10 +3562,10 @@
         <v>2</v>
       </c>
       <c r="C107" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D107" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E107">
         <v>250</v>
@@ -3588,10 +3588,10 @@
         <v>2</v>
       </c>
       <c r="C108" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D108" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E108">
         <v>251</v>
@@ -3614,10 +3614,10 @@
         <v>2</v>
       </c>
       <c r="C109" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D109" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E109">
         <v>169</v>
@@ -3640,10 +3640,10 @@
         <v>3</v>
       </c>
       <c r="C110" t="s">
+        <v>7</v>
+      </c>
+      <c r="D110" t="s">
         <v>8</v>
-      </c>
-      <c r="D110" t="s">
-        <v>9</v>
       </c>
       <c r="E110">
         <v>169</v>
@@ -3666,10 +3666,10 @@
         <v>3</v>
       </c>
       <c r="C111" t="s">
+        <v>9</v>
+      </c>
+      <c r="D111" t="s">
         <v>10</v>
-      </c>
-      <c r="D111" t="s">
-        <v>11</v>
       </c>
       <c r="E111">
         <v>169</v>
@@ -3692,10 +3692,10 @@
         <v>3</v>
       </c>
       <c r="C112" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D112" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E112">
         <v>169</v>
@@ -3718,10 +3718,10 @@
         <v>3</v>
       </c>
       <c r="C113" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D113" s="23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E113">
         <v>59</v>
@@ -3744,10 +3744,10 @@
         <v>3</v>
       </c>
       <c r="C114" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D114" s="23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E114">
         <v>60</v>
@@ -3770,10 +3770,10 @@
         <v>3</v>
       </c>
       <c r="C115" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D115" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E115">
         <v>61</v>
@@ -3796,10 +3796,10 @@
         <v>3</v>
       </c>
       <c r="C116" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D116" s="23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E116">
         <v>62</v>
@@ -3822,10 +3822,10 @@
         <v>3</v>
       </c>
       <c r="C117" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D117" s="23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E117">
         <v>63</v>
@@ -3848,10 +3848,10 @@
         <v>3</v>
       </c>
       <c r="C118" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D118" s="23" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E118">
         <v>64</v>
@@ -3874,10 +3874,10 @@
         <v>3</v>
       </c>
       <c r="C119" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D119" s="23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E119">
         <v>65</v>
@@ -3900,10 +3900,10 @@
         <v>3</v>
       </c>
       <c r="C120" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D120" s="23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E120">
         <v>66</v>
@@ -3926,10 +3926,10 @@
         <v>3</v>
       </c>
       <c r="C121" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D121" s="23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E121">
         <v>67</v>
@@ -3952,10 +3952,10 @@
         <v>3</v>
       </c>
       <c r="C122" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D122" s="23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E122">
         <v>68</v>
@@ -3978,10 +3978,10 @@
         <v>3</v>
       </c>
       <c r="C123" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D123" s="23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E123">
         <v>69</v>
@@ -4004,10 +4004,10 @@
         <v>3</v>
       </c>
       <c r="C124" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D124" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E124">
         <v>127</v>
@@ -4030,10 +4030,10 @@
         <v>3</v>
       </c>
       <c r="C125" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D125" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E125">
         <v>163</v>
@@ -4056,10 +4056,10 @@
         <v>3</v>
       </c>
       <c r="C126" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D126" s="23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E126">
         <v>164</v>
@@ -4082,10 +4082,10 @@
         <v>3</v>
       </c>
       <c r="C127" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D127" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E127">
         <v>165</v>
@@ -4108,10 +4108,10 @@
         <v>3</v>
       </c>
       <c r="C128" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D128" s="23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E128">
         <v>166</v>
@@ -4134,10 +4134,10 @@
         <v>3</v>
       </c>
       <c r="C129" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D129" s="23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E129">
         <v>167</v>
@@ -4160,10 +4160,10 @@
         <v>3</v>
       </c>
       <c r="C130" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D130" s="23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E130">
         <v>170</v>
@@ -4186,10 +4186,10 @@
         <v>3</v>
       </c>
       <c r="C131" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D131" s="23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E131">
         <v>219</v>
@@ -4212,10 +4212,10 @@
         <v>3</v>
       </c>
       <c r="C132" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D132" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E132">
         <v>221</v>
@@ -4238,10 +4238,10 @@
         <v>3</v>
       </c>
       <c r="C133" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D133" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E133">
         <v>222</v>
@@ -4264,10 +4264,10 @@
         <v>3</v>
       </c>
       <c r="C134" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D134" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E134">
         <v>223</v>
@@ -4290,10 +4290,10 @@
         <v>3</v>
       </c>
       <c r="C135" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D135" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E135">
         <v>224</v>
@@ -4316,10 +4316,10 @@
         <v>3</v>
       </c>
       <c r="C136" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D136" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E136">
         <v>225</v>
@@ -4342,10 +4342,10 @@
         <v>3</v>
       </c>
       <c r="C137" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D137" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E137">
         <v>226</v>
@@ -4368,10 +4368,10 @@
         <v>3</v>
       </c>
       <c r="C138" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D138" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E138">
         <v>227</v>
@@ -4394,10 +4394,10 @@
         <v>3</v>
       </c>
       <c r="C139" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D139" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E139">
         <v>228</v>
@@ -4420,10 +4420,10 @@
         <v>3</v>
       </c>
       <c r="C140" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D140" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E140">
         <v>229</v>
@@ -4446,10 +4446,10 @@
         <v>3</v>
       </c>
       <c r="C141" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D141" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E141">
         <v>230</v>
@@ -4472,10 +4472,10 @@
         <v>3</v>
       </c>
       <c r="C142" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D142" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E142">
         <v>231</v>
@@ -4498,10 +4498,10 @@
         <v>3</v>
       </c>
       <c r="C143" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D143" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E143">
         <v>232</v>
@@ -4524,10 +4524,10 @@
         <v>3</v>
       </c>
       <c r="C144" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D144" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E144">
         <v>233</v>
@@ -4550,10 +4550,10 @@
         <v>3</v>
       </c>
       <c r="C145" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D145" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E145">
         <v>234</v>
@@ -4576,10 +4576,10 @@
         <v>3</v>
       </c>
       <c r="C146" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D146" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E146">
         <v>235</v>
@@ -4602,10 +4602,10 @@
         <v>3</v>
       </c>
       <c r="C147" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D147" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E147">
         <v>236</v>
@@ -4628,10 +4628,10 @@
         <v>3</v>
       </c>
       <c r="C148" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D148" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E148">
         <v>237</v>
@@ -4654,10 +4654,10 @@
         <v>3</v>
       </c>
       <c r="C149" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D149" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E149">
         <v>238</v>
@@ -4680,10 +4680,10 @@
         <v>3</v>
       </c>
       <c r="C150" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D150" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E150">
         <v>239</v>
@@ -4706,10 +4706,10 @@
         <v>3</v>
       </c>
       <c r="C151" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D151" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E151">
         <v>240</v>
@@ -4732,10 +4732,10 @@
         <v>3</v>
       </c>
       <c r="C152" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D152" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E152">
         <v>241</v>
@@ -4758,10 +4758,10 @@
         <v>3</v>
       </c>
       <c r="C153" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D153" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E153">
         <v>242</v>
@@ -4784,10 +4784,10 @@
         <v>3</v>
       </c>
       <c r="C154" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D154" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E154">
         <v>243</v>
@@ -4810,10 +4810,10 @@
         <v>3</v>
       </c>
       <c r="C155" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D155" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E155">
         <v>244</v>
@@ -4836,10 +4836,10 @@
         <v>3</v>
       </c>
       <c r="C156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D156" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E156">
         <v>245</v>
@@ -4862,10 +4862,10 @@
         <v>3</v>
       </c>
       <c r="C157" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D157" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E157">
         <v>246</v>
@@ -4888,10 +4888,10 @@
         <v>3</v>
       </c>
       <c r="C158" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D158" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E158">
         <v>247</v>
@@ -4914,10 +4914,10 @@
         <v>3</v>
       </c>
       <c r="C159" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D159" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E159">
         <v>248</v>
@@ -4940,10 +4940,10 @@
         <v>3</v>
       </c>
       <c r="C160" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D160" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E160">
         <v>249</v>
@@ -4966,10 +4966,10 @@
         <v>3</v>
       </c>
       <c r="C161" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D161" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E161">
         <v>250</v>
@@ -4992,10 +4992,10 @@
         <v>3</v>
       </c>
       <c r="C162" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D162" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E162">
         <v>251</v>
@@ -5018,10 +5018,10 @@
         <v>3</v>
       </c>
       <c r="C163" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D163" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E163">
         <v>169</v>

</xml_diff>